<commit_message>
Add gridlines to TOTAL RH sheet
Native gridlines are off on this sheet; add a thin border to every
populated/filled cell across all sections (weekly blocks, remarks,
mini roll-up, durian table, year x brand x size matrix) so each
table is ruled without bordering the blank gap rows/columns between
them.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_9-21.xlsx
+++ b/Stock_Daily_Reefer_9-21.xlsx
@@ -251,7 +251,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -286,6 +286,83 @@
       <bottom style="thin">
         <color rgb="00D9D9D9"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -335,55 +412,56 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -408,9 +486,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -453,14 +528,17 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -3335,6 +3413,16 @@
         <f>"Stock vs Booking Report - Reefer (20'RE / 40'RH)  as of "&amp;DAY(Control!$B$1)&amp;" "&amp;CHOOSE(MONTH(Control!$B$1),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;" "&amp;YEAR(Control!$B$1)</f>
         <v/>
       </c>
+      <c r="B1" s="51" t="n"/>
+      <c r="C1" s="51" t="n"/>
+      <c r="D1" s="51" t="n"/>
+      <c r="E1" s="51" t="n"/>
+      <c r="F1" s="51" t="n"/>
+      <c r="G1" s="51" t="n"/>
+      <c r="H1" s="51" t="n"/>
+      <c r="I1" s="51" t="n"/>
+      <c r="J1" s="51" t="n"/>
+      <c r="K1" s="52" t="n"/>
       <c r="L1" s="1" t="n"/>
       <c r="M1" s="1" t="n"/>
       <c r="N1" s="1" t="n"/>
@@ -3348,6 +3436,8 @@
           <t>BKK27 / BC2</t>
         </is>
       </c>
+      <c r="C2" s="51" t="n"/>
+      <c r="D2" s="52" t="n"/>
       <c r="E2" s="1" t="n"/>
       <c r="F2" s="1" t="n"/>
       <c r="G2" s="1" t="n"/>
@@ -3356,6 +3446,8 @@
           <t>LCH27 / HAST</t>
         </is>
       </c>
+      <c r="I2" s="51" t="n"/>
+      <c r="J2" s="52" t="n"/>
       <c r="K2" s="1" t="n"/>
       <c r="L2" s="1" t="n"/>
       <c r="M2" s="5" t="inlineStr">
@@ -3412,16 +3504,16 @@
       </c>
       <c r="K3" s="1" t="n"/>
       <c r="L3" s="1" t="n"/>
-      <c r="M3" s="1" t="inlineStr">
+      <c r="M3" s="7" t="inlineStr">
         <is>
           <t>BC</t>
         </is>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="8">
         <f>C4</f>
         <v/>
       </c>
-      <c r="O3" s="7">
+      <c r="O3" s="8">
         <f>D4</f>
         <v/>
       </c>
@@ -3429,88 +3521,88 @@
     </row>
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="1" t="n"/>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Stock empty in yard</t>
         </is>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="10" t="n">
         <v>20</v>
       </c>
       <c r="E4" s="1" t="n"/>
       <c r="F4" s="1" t="n"/>
       <c r="G4" s="1" t="n"/>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>Stock empty in yard</t>
         </is>
       </c>
-      <c r="I4" s="9" t="n">
+      <c r="I4" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="J4" s="9" t="n">
+      <c r="J4" s="10" t="n">
         <v>46</v>
       </c>
       <c r="K4" s="1" t="n"/>
       <c r="L4" s="1" t="n"/>
-      <c r="M4" s="1" t="inlineStr">
+      <c r="M4" s="7" t="inlineStr">
         <is>
           <t>HAST</t>
         </is>
       </c>
-      <c r="N4" s="7">
+      <c r="N4" s="8">
         <f>I4</f>
         <v/>
       </c>
-      <c r="O4" s="7">
+      <c r="O4" s="8">
         <f>J4</f>
         <v/>
       </c>
       <c r="P4" s="1" t="n"/>
     </row>
     <row r="5" ht="13" customHeight="1">
-      <c r="A5" s="1">
+      <c r="A5" s="7">
         <f>Control!$A$4</f>
         <v/>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Booking Pending pick up</t>
         </is>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&lt;"&amp;Control!$B$1)</f>
         <v/>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&lt;"&amp;Control!$B$1)</f>
         <v/>
       </c>
       <c r="E5" s="1" t="n"/>
       <c r="F5" s="1" t="n"/>
-      <c r="G5" s="1">
+      <c r="G5" s="7">
         <f>Control!$A$4</f>
         <v/>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Booking Pending pick up</t>
         </is>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&lt;"&amp;Control!$B$1)</f>
         <v/>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&lt;"&amp;Control!$B$1)</f>
         <v/>
       </c>
       <c r="K5" s="1" t="n"/>
       <c r="L5" s="1" t="n"/>
-      <c r="M5" s="10" t="inlineStr">
+      <c r="M5" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -3526,37 +3618,37 @@
       <c r="P5" s="1" t="n"/>
     </row>
     <row r="6" ht="13" customHeight="1">
-      <c r="A6" s="1">
+      <c r="A6" s="7">
         <f>Control!$A$4</f>
         <v/>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="7">
         <f>"Booking on "&amp;DAY(Control!$B$1)&amp;" "&amp;CHOOSE(MONTH(Control!$B$1),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"="&amp;Control!$B$1)</f>
         <v/>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"="&amp;Control!$B$1)</f>
         <v/>
       </c>
       <c r="E6" s="1" t="n"/>
       <c r="F6" s="1" t="n"/>
-      <c r="G6" s="1">
+      <c r="G6" s="7">
         <f>Control!$A$4</f>
         <v/>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="7">
         <f>"Booking on "&amp;DAY(Control!$B$1)&amp;" "&amp;CHOOSE(MONTH(Control!$B$1),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"="&amp;Control!$B$1)</f>
         <v/>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"="&amp;Control!$B$1)</f>
         <v/>
       </c>
@@ -3568,37 +3660,37 @@
       <c r="P6" s="1" t="n"/>
     </row>
     <row r="7" ht="13" customHeight="1">
-      <c r="A7" s="1">
+      <c r="A7" s="7">
         <f>Control!$A$4</f>
         <v/>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="7">
         <f>"Booking on "&amp;IF(Control!$B$9=Control!$C$4,DAY(Control!$B$9)&amp;" "&amp;CHOOSE(MONTH(Control!$B$9),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),IF(MONTH(Control!$B$9)=MONTH(Control!$C$4),DAY(Control!$B$9)&amp;"-"&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),DAY(Control!$B$9)&amp;" "&amp;CHOOSE(MONTH(Control!$B$9),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;"-"&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")))</f>
         <v/>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B$9,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C$4)</f>
         <v/>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B$9,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C$4)</f>
         <v/>
       </c>
       <c r="E7" s="1" t="n"/>
       <c r="F7" s="1" t="n"/>
-      <c r="G7" s="1">
+      <c r="G7" s="7">
         <f>Control!$A$4</f>
         <v/>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="7">
         <f>"Booking on "&amp;IF(Control!$B$9=Control!$C$4,DAY(Control!$B$9)&amp;" "&amp;CHOOSE(MONTH(Control!$B$9),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),IF(MONTH(Control!$B$9)=MONTH(Control!$C$4),DAY(Control!$B$9)&amp;"-"&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),DAY(Control!$B$9)&amp;" "&amp;CHOOSE(MONTH(Control!$B$9),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;"-"&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")))</f>
         <v/>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B$9,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C$4)</f>
         <v/>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B$9,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C$4)</f>
         <v/>
       </c>
@@ -3623,97 +3715,97 @@
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="1" t="n"/>
-      <c r="B8" s="11">
+      <c r="B8" s="12">
         <f>"AV Balance till "&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C8" s="51">
+      <c r="C8" s="53">
         <f>C4-C5-C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="52">
+      <c r="D8" s="54">
         <f>D4-D5-D6-D7</f>
         <v/>
       </c>
       <c r="E8" s="1" t="n"/>
       <c r="F8" s="1" t="n"/>
       <c r="G8" s="1" t="n"/>
-      <c r="H8" s="11">
+      <c r="H8" s="12">
         <f>"AV Balance till "&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I8" s="51">
+      <c r="I8" s="53">
         <f>I4-I5-I6-I7</f>
         <v/>
       </c>
-      <c r="J8" s="51">
+      <c r="J8" s="53">
         <f>J4-J5-J6-J7</f>
         <v/>
       </c>
       <c r="K8" s="1" t="n"/>
       <c r="L8" s="1" t="n"/>
-      <c r="M8" s="1" t="inlineStr">
+      <c r="M8" s="7" t="inlineStr">
         <is>
           <t>BC</t>
         </is>
       </c>
-      <c r="N8" s="7">
+      <c r="N8" s="8">
         <f>C5+C6+C7+C9+C11</f>
         <v/>
       </c>
-      <c r="O8" s="7">
+      <c r="O8" s="8">
         <f>D5+D6+D7+D9+D11</f>
         <v/>
       </c>
       <c r="P8" s="1" t="n"/>
     </row>
     <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="1">
+      <c r="A9" s="7">
         <f>Control!$A$5</f>
         <v/>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="7">
         <f>"Booking on "&amp;IF(Control!$B5=Control!$C5,DAY(Control!$B5)&amp;" "&amp;CHOOSE(MONTH(Control!$B5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),IF(MONTH(Control!$B5)=MONTH(Control!$C5),DAY(Control!$B5)&amp;"-"&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),DAY(Control!$B5)&amp;" "&amp;CHOOSE(MONTH(Control!$B5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;"-"&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")))</f>
         <v/>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B5,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C5)</f>
         <v/>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B5,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C5)</f>
         <v/>
       </c>
       <c r="E9" s="1" t="n"/>
       <c r="F9" s="1" t="n"/>
-      <c r="G9" s="1">
+      <c r="G9" s="7">
         <f>Control!$A$5</f>
         <v/>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="7">
         <f>"Booking on "&amp;IF(Control!$B5=Control!$C5,DAY(Control!$B5)&amp;" "&amp;CHOOSE(MONTH(Control!$B5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),IF(MONTH(Control!$B5)=MONTH(Control!$C5),DAY(Control!$B5)&amp;"-"&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),DAY(Control!$B5)&amp;" "&amp;CHOOSE(MONTH(Control!$B5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;"-"&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")))</f>
         <v/>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B5,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C5)</f>
         <v/>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B5,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C5)</f>
         <v/>
       </c>
       <c r="K9" s="1" t="n"/>
       <c r="L9" s="1" t="n"/>
-      <c r="M9" s="1" t="inlineStr">
+      <c r="M9" s="7" t="inlineStr">
         <is>
           <t>HAST</t>
         </is>
       </c>
-      <c r="N9" s="7">
+      <c r="N9" s="8">
         <f>I5+I6+I7+I9+I11</f>
         <v/>
       </c>
-      <c r="O9" s="7">
+      <c r="O9" s="8">
         <f>J5+J6+J7+J9+J11</f>
         <v/>
       </c>
@@ -3721,36 +3813,36 @@
     </row>
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="11">
+      <c r="B10" s="12">
         <f>"AV Balance till "&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C10" s="51">
+      <c r="C10" s="53">
         <f>C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="52">
+      <c r="D10" s="54">
         <f>D8-D9</f>
         <v/>
       </c>
       <c r="E10" s="1" t="n"/>
       <c r="F10" s="1" t="n"/>
       <c r="G10" s="1" t="n"/>
-      <c r="H10" s="11">
+      <c r="H10" s="12">
         <f>"AV Balance till "&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I10" s="51">
+      <c r="I10" s="53">
         <f>I8-I9</f>
         <v/>
       </c>
-      <c r="J10" s="51">
+      <c r="J10" s="53">
         <f>J8-J9</f>
         <v/>
       </c>
       <c r="K10" s="1" t="n"/>
       <c r="L10" s="1" t="n"/>
-      <c r="M10" s="10" t="inlineStr">
+      <c r="M10" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -3766,37 +3858,37 @@
       <c r="P10" s="1" t="n"/>
     </row>
     <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="1">
+      <c r="A11" s="7">
         <f>Control!$A$6</f>
         <v/>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="7">
         <f>"Booking on "&amp;IF(Control!$B6=Control!$C6,DAY(Control!$B6)&amp;" "&amp;CHOOSE(MONTH(Control!$B6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),IF(MONTH(Control!$B6)=MONTH(Control!$C6),DAY(Control!$B6)&amp;"-"&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),DAY(Control!$B6)&amp;" "&amp;CHOOSE(MONTH(Control!$B6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;"-"&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")))</f>
         <v/>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B6,BookingRaw!$B$2:$B$8000,"&lt;="&amp;DATE(2026,10,18))</f>
         <v/>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B6,BookingRaw!$B$2:$B$8000,"&lt;="&amp;DATE(2026,10,18))</f>
         <v/>
       </c>
       <c r="E11" s="1" t="n"/>
       <c r="F11" s="1" t="n"/>
-      <c r="G11" s="1">
+      <c r="G11" s="7">
         <f>Control!$A$6</f>
         <v/>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="7">
         <f>"Booking on "&amp;IF(Control!$B6=Control!$C6,DAY(Control!$B6)&amp;" "&amp;CHOOSE(MONTH(Control!$B6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),IF(MONTH(Control!$B6)=MONTH(Control!$C6),DAY(Control!$B6)&amp;"-"&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),DAY(Control!$B6)&amp;" "&amp;CHOOSE(MONTH(Control!$B6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;"-"&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")))</f>
         <v/>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="7">
         <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B6,BookingRaw!$B$2:$B$8000,"&lt;="&amp;DATE(2026,10,18))</f>
         <v/>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="7">
         <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B6,BookingRaw!$B$2:$B$8000,"&lt;="&amp;DATE(2026,10,18))</f>
         <v/>
       </c>
@@ -3809,30 +3901,30 @@
     </row>
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="11">
+      <c r="B12" s="12">
         <f>"AV Balance till "&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C12" s="51">
+      <c r="C12" s="53">
         <f>C10-C11</f>
         <v/>
       </c>
-      <c r="D12" s="52">
+      <c r="D12" s="54">
         <f>D10-D11</f>
         <v/>
       </c>
       <c r="E12" s="1" t="n"/>
       <c r="F12" s="1" t="n"/>
       <c r="G12" s="1" t="n"/>
-      <c r="H12" s="11">
+      <c r="H12" s="12">
         <f>"AV Balance till "&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I12" s="51">
+      <c r="I12" s="53">
         <f>I10-I11</f>
         <v/>
       </c>
-      <c r="J12" s="52">
+      <c r="J12" s="54">
         <f>J10-J11</f>
         <v/>
       </c>
@@ -3868,28 +3960,28 @@
       <c r="J13" s="1" t="n"/>
       <c r="K13" s="1" t="n"/>
       <c r="L13" s="1" t="n"/>
-      <c r="M13" s="1" t="inlineStr">
+      <c r="M13" s="7" t="inlineStr">
         <is>
           <t>BC</t>
         </is>
       </c>
-      <c r="N13" s="7">
+      <c r="N13" s="8">
         <f>C12</f>
         <v/>
       </c>
-      <c r="O13" s="7">
+      <c r="O13" s="8">
         <f>D12</f>
         <v/>
       </c>
       <c r="P13" s="1" t="n"/>
     </row>
     <row r="14" ht="13" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Remarks:</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>AV = stock with move code IED / IEP / IER (available)   |   DMG = move code OER (damaged)</t>
         </is>
@@ -3904,16 +3996,16 @@
       <c r="J14" s="1" t="n"/>
       <c r="K14" s="1" t="n"/>
       <c r="L14" s="1" t="n"/>
-      <c r="M14" s="1" t="inlineStr">
+      <c r="M14" s="7" t="inlineStr">
         <is>
           <t>HAST</t>
         </is>
       </c>
-      <c r="N14" s="7">
+      <c r="N14" s="8">
         <f>I12</f>
         <v/>
       </c>
-      <c r="O14" s="7">
+      <c r="O14" s="8">
         <f>J12</f>
         <v/>
       </c>
@@ -3948,7 +4040,7 @@
       </c>
       <c r="K15" s="1" t="n"/>
       <c r="L15" s="1" t="n"/>
-      <c r="M15" s="10" t="inlineStr">
+      <c r="M15" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -3965,32 +4057,32 @@
     </row>
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="1" t="n"/>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>AV</t>
         </is>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="8">
         <f>COUNTIFS(StockRaw!$A$2:$A$101,"BKK27",StockRaw!$B$2:$B$101,"22RE",StockRaw!$C$2:$C$101,"IED")+COUNTIFS(StockRaw!$A$2:$A$101,"BKK27",StockRaw!$B$2:$B$101,"22RE",StockRaw!$C$2:$C$101,"IEP")+COUNTIFS(StockRaw!$A$2:$A$101,"BKK27",StockRaw!$B$2:$B$101,"22RE",StockRaw!$C$2:$C$101,"IER")</f>
         <v/>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="8">
         <f>COUNTIFS(StockRaw!$A$2:$A$101,"BKK27",StockRaw!$B$2:$B$101,"45RE",StockRaw!$C$2:$C$101,"IED")+COUNTIFS(StockRaw!$A$2:$A$101,"BKK27",StockRaw!$B$2:$B$101,"45RE",StockRaw!$C$2:$C$101,"IEP")+COUNTIFS(StockRaw!$A$2:$A$101,"BKK27",StockRaw!$B$2:$B$101,"45RE",StockRaw!$C$2:$C$101,"IER")</f>
         <v/>
       </c>
       <c r="E16" s="1" t="n"/>
       <c r="F16" s="1" t="n"/>
       <c r="G16" s="1" t="n"/>
-      <c r="H16" s="15" t="inlineStr">
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>AV</t>
         </is>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="8">
         <f>COUNTIFS(StockRaw!$A$2:$A$101,"LCH27",StockRaw!$B$2:$B$101,"22RE",StockRaw!$C$2:$C$101,"IED")+COUNTIFS(StockRaw!$A$2:$A$101,"LCH27",StockRaw!$B$2:$B$101,"22RE",StockRaw!$C$2:$C$101,"IEP")+COUNTIFS(StockRaw!$A$2:$A$101,"LCH27",StockRaw!$B$2:$B$101,"22RE",StockRaw!$C$2:$C$101,"IER")</f>
         <v/>
       </c>
-      <c r="J16" s="7">
+      <c r="J16" s="8">
         <f>COUNTIFS(StockRaw!$A$2:$A$101,"LCH27",StockRaw!$B$2:$B$101,"45RE",StockRaw!$C$2:$C$101,"IED")+COUNTIFS(StockRaw!$A$2:$A$101,"LCH27",StockRaw!$B$2:$B$101,"45RE",StockRaw!$C$2:$C$101,"IEP")+COUNTIFS(StockRaw!$A$2:$A$101,"LCH27",StockRaw!$B$2:$B$101,"45RE",StockRaw!$C$2:$C$101,"IER")</f>
         <v/>
       </c>
@@ -4003,32 +4095,32 @@
     </row>
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="1" t="n"/>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>DMG</t>
         </is>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="8">
         <f>COUNTIFS(StockRaw!$A$2:$A$101,"BKK27",StockRaw!$B$2:$B$101,"22RE",StockRaw!$C$2:$C$101,"OER")</f>
         <v/>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="8">
         <f>COUNTIFS(StockRaw!$A$2:$A$101,"BKK27",StockRaw!$B$2:$B$101,"45RE",StockRaw!$C$2:$C$101,"OER")</f>
         <v/>
       </c>
       <c r="E17" s="1" t="n"/>
       <c r="F17" s="1" t="n"/>
       <c r="G17" s="1" t="n"/>
-      <c r="H17" s="15" t="inlineStr">
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>DMG</t>
         </is>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="8">
         <f>COUNTIFS(StockRaw!$A$2:$A$101,"LCH27",StockRaw!$B$2:$B$101,"22RE",StockRaw!$C$2:$C$101,"OER")</f>
         <v/>
       </c>
-      <c r="J17" s="7">
+      <c r="J17" s="8">
         <f>COUNTIFS(StockRaw!$A$2:$A$101,"LCH27",StockRaw!$B$2:$B$101,"45RE",StockRaw!$C$2:$C$101,"OER")</f>
         <v/>
       </c>
@@ -4077,18 +4169,24 @@
     </row>
     <row r="20" ht="13" customHeight="1">
       <c r="A20" s="1" t="n"/>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>BKK / BC2 (BKK27)</t>
         </is>
       </c>
+      <c r="C20" s="51" t="n"/>
+      <c r="D20" s="51" t="n"/>
+      <c r="E20" s="52" t="n"/>
       <c r="F20" s="1" t="n"/>
       <c r="G20" s="1" t="n"/>
-      <c r="H20" s="16" t="inlineStr">
+      <c r="H20" s="17" t="inlineStr">
         <is>
           <t>LCH / HAST (LCH27)</t>
         </is>
       </c>
+      <c r="I20" s="51" t="n"/>
+      <c r="J20" s="51" t="n"/>
+      <c r="K20" s="52" t="n"/>
       <c r="L20" s="1" t="n"/>
       <c r="M20" s="1" t="n"/>
       <c r="N20" s="1" t="n"/>
@@ -4097,7 +4195,7 @@
     </row>
     <row r="21" ht="13" customHeight="1">
       <c r="A21" s="1" t="n"/>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>YEAR BUILT 5 YEARS
 FOR DURIAN SEASON</t>
@@ -4120,7 +4218,7 @@
       </c>
       <c r="F21" s="1" t="n"/>
       <c r="G21" s="1" t="n"/>
-      <c r="H21" s="17" t="inlineStr">
+      <c r="H21" s="18" t="inlineStr">
         <is>
           <t>YEAR BUILT 5 YEARS
 FOR DURIAN SEASON</t>
@@ -4149,6 +4247,7 @@
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="1" t="n"/>
+      <c r="B22" s="55" t="n"/>
       <c r="C22" s="4" t="inlineStr">
         <is>
           <t>45RE</t>
@@ -4166,6 +4265,7 @@
       </c>
       <c r="F22" s="1" t="n"/>
       <c r="G22" s="1" t="n"/>
+      <c r="H22" s="55" t="n"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
           <t>45RE</t>
@@ -4189,30 +4289,30 @@
     </row>
     <row r="23" ht="13" customHeight="1">
       <c r="A23" s="1" t="n"/>
-      <c r="B23" s="7" t="n">
+      <c r="B23" s="8" t="n">
         <v>2026</v>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="7" t="n">
+      <c r="E23" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="1" t="n"/>
       <c r="G23" s="1" t="n"/>
-      <c r="H23" s="7" t="n">
+      <c r="H23" s="8" t="n">
         <v>2026</v>
       </c>
-      <c r="I23" s="7" t="n">
+      <c r="I23" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J23" s="7" t="n">
+      <c r="J23" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="7" t="n">
+      <c r="K23" s="8" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="1" t="n"/>
@@ -4223,30 +4323,30 @@
     </row>
     <row r="24" ht="13" customHeight="1">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="7" t="n">
+      <c r="B24" s="8" t="n">
         <v>2025</v>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E24" s="7" t="n">
+      <c r="E24" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="1" t="n"/>
       <c r="G24" s="1" t="n"/>
-      <c r="H24" s="7" t="n">
+      <c r="H24" s="8" t="n">
         <v>2025</v>
       </c>
-      <c r="I24" s="7" t="n">
+      <c r="I24" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="J24" s="7" t="n">
+      <c r="J24" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="7" t="n">
+      <c r="K24" s="8" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="1" t="n"/>
@@ -4257,30 +4357,30 @@
     </row>
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="7" t="n">
+      <c r="B25" s="8" t="n">
         <v>2024</v>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C25" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="D25" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="7" t="n">
+      <c r="E25" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="1" t="n"/>
       <c r="G25" s="1" t="n"/>
-      <c r="H25" s="7" t="n">
+      <c r="H25" s="8" t="n">
         <v>2024</v>
       </c>
-      <c r="I25" s="7" t="n">
+      <c r="I25" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J25" s="7" t="n">
+      <c r="J25" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="7" t="n">
+      <c r="K25" s="8" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="1" t="n"/>
@@ -4291,30 +4391,30 @@
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="7" t="n">
+      <c r="B26" s="8" t="n">
         <v>2023</v>
       </c>
-      <c r="C26" s="7" t="n">
+      <c r="C26" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="7" t="n">
+      <c r="D26" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="7" t="n">
+      <c r="E26" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="1" t="n"/>
       <c r="G26" s="1" t="n"/>
-      <c r="H26" s="7" t="n">
+      <c r="H26" s="8" t="n">
         <v>2023</v>
       </c>
-      <c r="I26" s="7" t="n">
+      <c r="I26" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="J26" s="7" t="n">
+      <c r="J26" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="7" t="n">
+      <c r="K26" s="8" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="1" t="n"/>
@@ -4325,30 +4425,30 @@
     </row>
     <row r="27" ht="13" customHeight="1">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="7" t="n">
+      <c r="B27" s="8" t="n">
         <v>2022</v>
       </c>
-      <c r="C27" s="7" t="n">
+      <c r="C27" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="7" t="n">
+      <c r="D27" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E27" s="7" t="n">
+      <c r="E27" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="1" t="n"/>
       <c r="G27" s="1" t="n"/>
-      <c r="H27" s="7" t="n">
+      <c r="H27" s="8" t="n">
         <v>2022</v>
       </c>
-      <c r="I27" s="7" t="n">
+      <c r="I27" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J27" s="7" t="n">
+      <c r="J27" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="K27" s="7" t="n">
+      <c r="K27" s="8" t="n">
         <v>0</v>
       </c>
       <c r="L27" s="1" t="n"/>
@@ -4359,30 +4459,30 @@
     </row>
     <row r="28" ht="13" customHeight="1">
       <c r="A28" s="1" t="n"/>
-      <c r="B28" s="7" t="n">
+      <c r="B28" s="8" t="n">
         <v>2021</v>
       </c>
-      <c r="C28" s="7" t="n">
+      <c r="C28" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="D28" s="7" t="n">
+      <c r="D28" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="7" t="n">
+      <c r="E28" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="1" t="n"/>
       <c r="G28" s="1" t="n"/>
-      <c r="H28" s="7" t="n">
+      <c r="H28" s="8" t="n">
         <v>2021</v>
       </c>
-      <c r="I28" s="7" t="n">
+      <c r="I28" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="J28" s="7" t="n">
+      <c r="J28" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="7" t="n">
+      <c r="K28" s="8" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="1" t="n"/>
@@ -4433,24 +4533,24 @@
       <c r="A30" s="1" t="n"/>
       <c r="B30" s="1" t="n"/>
       <c r="C30" s="1" t="n"/>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>OVER 5 Y</t>
         </is>
       </c>
-      <c r="E30" s="19" t="n">
+      <c r="E30" s="20" t="n">
         <v>11</v>
       </c>
       <c r="F30" s="1" t="n"/>
       <c r="G30" s="1" t="n"/>
       <c r="H30" s="1" t="n"/>
       <c r="I30" s="1" t="n"/>
-      <c r="J30" s="18" t="inlineStr">
+      <c r="J30" s="19" t="inlineStr">
         <is>
           <t>OVER 5 Y</t>
         </is>
       </c>
-      <c r="K30" s="19" t="n">
+      <c r="K30" s="20" t="n">
         <v>29</v>
       </c>
       <c r="L30" s="1" t="n"/>
@@ -4502,16 +4602,28 @@
           <t>BKK27 / BC2  —  Stock by Built Year x Brand x Size</t>
         </is>
       </c>
+      <c r="C33" s="51" t="n"/>
+      <c r="D33" s="51" t="n"/>
+      <c r="E33" s="51" t="n"/>
+      <c r="F33" s="51" t="n"/>
+      <c r="G33" s="51" t="n"/>
+      <c r="H33" s="52" t="n"/>
       <c r="I33" s="1" t="n"/>
       <c r="J33" s="3" t="inlineStr">
         <is>
           <t>LCH27 / HAST  —  Stock by Built Year x Brand x Size</t>
         </is>
       </c>
+      <c r="K33" s="51" t="n"/>
+      <c r="L33" s="51" t="n"/>
+      <c r="M33" s="51" t="n"/>
+      <c r="N33" s="51" t="n"/>
+      <c r="O33" s="51" t="n"/>
+      <c r="P33" s="52" t="n"/>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="1" t="n"/>
-      <c r="B34" s="17" t="inlineStr">
+      <c r="B34" s="18" t="inlineStr">
         <is>
           <t>YEAR
 BUILT</t>
@@ -4522,18 +4634,21 @@
           <t>CARRIER</t>
         </is>
       </c>
+      <c r="D34" s="52" t="n"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
           <t>DAIKIN</t>
         </is>
       </c>
+      <c r="F34" s="52" t="n"/>
       <c r="G34" s="4" t="inlineStr">
         <is>
           <t>THERMO KING</t>
         </is>
       </c>
+      <c r="H34" s="52" t="n"/>
       <c r="I34" s="1" t="n"/>
-      <c r="J34" s="17" t="inlineStr">
+      <c r="J34" s="18" t="inlineStr">
         <is>
           <t>YEAR
 BUILT</t>
@@ -4544,76 +4659,81 @@
           <t>CARRIER</t>
         </is>
       </c>
+      <c r="L34" s="52" t="n"/>
       <c r="M34" s="4" t="inlineStr">
         <is>
           <t>DAIKIN</t>
         </is>
       </c>
+      <c r="N34" s="52" t="n"/>
       <c r="O34" s="4" t="inlineStr">
         <is>
           <t>THERMO KING</t>
         </is>
       </c>
+      <c r="P34" s="52" t="n"/>
     </row>
     <row r="35" ht="13" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="C35" s="21" t="inlineStr">
+      <c r="B35" s="55" t="n"/>
+      <c r="C35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="D35" s="21" t="inlineStr">
+      <c r="D35" s="22" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
       </c>
-      <c r="E35" s="21" t="inlineStr">
+      <c r="E35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="F35" s="21" t="inlineStr">
+      <c r="F35" s="22" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
       </c>
-      <c r="G35" s="21" t="inlineStr">
+      <c r="G35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="H35" s="21" t="inlineStr">
+      <c r="H35" s="22" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
       </c>
       <c r="I35" s="1" t="n"/>
-      <c r="K35" s="21" t="inlineStr">
+      <c r="J35" s="55" t="n"/>
+      <c r="K35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="L35" s="21" t="inlineStr">
+      <c r="L35" s="22" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
       </c>
-      <c r="M35" s="21" t="inlineStr">
+      <c r="M35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="N35" s="21" t="inlineStr">
+      <c r="N35" s="22" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
       </c>
-      <c r="O35" s="21" t="inlineStr">
+      <c r="O35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="P35" s="21" t="inlineStr">
+      <c r="P35" s="22" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
@@ -4621,493 +4741,493 @@
     </row>
     <row r="36" ht="13" customHeight="1">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="22" t="n">
+      <c r="B36" s="23" t="n">
         <v>2026</v>
       </c>
-      <c r="C36" s="23" t="n"/>
-      <c r="D36" s="23" t="n"/>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="23" t="n"/>
-      <c r="G36" s="23" t="n"/>
-      <c r="H36" s="23" t="n"/>
+      <c r="C36" s="24" t="n"/>
+      <c r="D36" s="24" t="n"/>
+      <c r="E36" s="24" t="n"/>
+      <c r="F36" s="24" t="n"/>
+      <c r="G36" s="24" t="n"/>
+      <c r="H36" s="24" t="n"/>
       <c r="I36" s="1" t="n"/>
-      <c r="J36" s="22" t="n">
+      <c r="J36" s="23" t="n">
         <v>2026</v>
       </c>
-      <c r="K36" s="23" t="n"/>
-      <c r="L36" s="23" t="n"/>
-      <c r="M36" s="23" t="n"/>
-      <c r="N36" s="23" t="n"/>
-      <c r="O36" s="23" t="n"/>
-      <c r="P36" s="23" t="n"/>
+      <c r="K36" s="24" t="n"/>
+      <c r="L36" s="24" t="n"/>
+      <c r="M36" s="24" t="n"/>
+      <c r="N36" s="24" t="n"/>
+      <c r="O36" s="24" t="n"/>
+      <c r="P36" s="24" t="n"/>
     </row>
     <row r="37" ht="13" customHeight="1">
       <c r="A37" s="1" t="n"/>
-      <c r="B37" s="22" t="n">
+      <c r="B37" s="23" t="n">
         <v>2025</v>
       </c>
-      <c r="C37" s="23" t="n"/>
-      <c r="D37" s="23" t="n">
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="E37" s="23" t="n">
+      <c r="E37" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F37" s="23" t="n"/>
-      <c r="G37" s="23" t="n"/>
-      <c r="H37" s="23" t="n"/>
+      <c r="F37" s="24" t="n"/>
+      <c r="G37" s="24" t="n"/>
+      <c r="H37" s="24" t="n"/>
       <c r="I37" s="1" t="n"/>
-      <c r="J37" s="22" t="n">
+      <c r="J37" s="23" t="n">
         <v>2025</v>
       </c>
-      <c r="K37" s="23" t="n"/>
-      <c r="L37" s="23" t="n">
+      <c r="K37" s="24" t="n"/>
+      <c r="L37" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="M37" s="23" t="n">
+      <c r="M37" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="N37" s="23" t="n"/>
-      <c r="O37" s="23" t="n"/>
-      <c r="P37" s="23" t="n"/>
+      <c r="N37" s="24" t="n"/>
+      <c r="O37" s="24" t="n"/>
+      <c r="P37" s="24" t="n"/>
     </row>
     <row r="38" ht="13" customHeight="1">
       <c r="A38" s="1" t="n"/>
-      <c r="B38" s="22" t="n">
+      <c r="B38" s="23" t="n">
         <v>2024</v>
       </c>
-      <c r="C38" s="23" t="n"/>
-      <c r="D38" s="23" t="n"/>
-      <c r="E38" s="23" t="n"/>
-      <c r="F38" s="23" t="n"/>
-      <c r="G38" s="23" t="n"/>
-      <c r="H38" s="23" t="n"/>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="24" t="n"/>
+      <c r="G38" s="24" t="n"/>
+      <c r="H38" s="24" t="n"/>
       <c r="I38" s="1" t="n"/>
-      <c r="J38" s="22" t="n">
+      <c r="J38" s="23" t="n">
         <v>2024</v>
       </c>
-      <c r="K38" s="23" t="n"/>
-      <c r="L38" s="23" t="n"/>
-      <c r="M38" s="23" t="n"/>
-      <c r="N38" s="23" t="n"/>
-      <c r="O38" s="23" t="n"/>
-      <c r="P38" s="23" t="n"/>
+      <c r="K38" s="24" t="n"/>
+      <c r="L38" s="24" t="n"/>
+      <c r="M38" s="24" t="n"/>
+      <c r="N38" s="24" t="n"/>
+      <c r="O38" s="24" t="n"/>
+      <c r="P38" s="24" t="n"/>
     </row>
     <row r="39" ht="13" customHeight="1">
       <c r="A39" s="1" t="n"/>
-      <c r="B39" s="22" t="n">
+      <c r="B39" s="23" t="n">
         <v>2023</v>
       </c>
-      <c r="C39" s="23" t="n"/>
-      <c r="D39" s="23" t="n"/>
-      <c r="E39" s="23" t="n"/>
-      <c r="F39" s="23" t="n"/>
-      <c r="G39" s="23" t="n"/>
-      <c r="H39" s="23" t="n"/>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="24" t="n"/>
+      <c r="H39" s="24" t="n"/>
       <c r="I39" s="1" t="n"/>
-      <c r="J39" s="22" t="n">
+      <c r="J39" s="23" t="n">
         <v>2023</v>
       </c>
-      <c r="K39" s="23" t="n"/>
-      <c r="L39" s="23" t="n">
+      <c r="K39" s="24" t="n"/>
+      <c r="L39" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="M39" s="23" t="n"/>
-      <c r="N39" s="23" t="n"/>
-      <c r="O39" s="23" t="n"/>
-      <c r="P39" s="23" t="n"/>
+      <c r="M39" s="24" t="n"/>
+      <c r="N39" s="24" t="n"/>
+      <c r="O39" s="24" t="n"/>
+      <c r="P39" s="24" t="n"/>
     </row>
     <row r="40" ht="13" customHeight="1">
       <c r="A40" s="1" t="n"/>
-      <c r="B40" s="22" t="n">
+      <c r="B40" s="23" t="n">
         <v>2022</v>
       </c>
-      <c r="C40" s="23" t="n"/>
-      <c r="D40" s="23" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="24" t="n"/>
+      <c r="H40" s="24" t="n"/>
       <c r="I40" s="1" t="n"/>
-      <c r="J40" s="22" t="n">
+      <c r="J40" s="23" t="n">
         <v>2022</v>
       </c>
-      <c r="K40" s="23" t="n"/>
-      <c r="L40" s="23" t="n"/>
-      <c r="M40" s="23" t="n"/>
-      <c r="N40" s="23" t="n"/>
-      <c r="O40" s="23" t="n"/>
-      <c r="P40" s="23" t="n"/>
+      <c r="K40" s="24" t="n"/>
+      <c r="L40" s="24" t="n"/>
+      <c r="M40" s="24" t="n"/>
+      <c r="N40" s="24" t="n"/>
+      <c r="O40" s="24" t="n"/>
+      <c r="P40" s="24" t="n"/>
     </row>
     <row r="41" ht="13" customHeight="1">
       <c r="A41" s="1" t="n"/>
-      <c r="B41" s="22" t="n">
+      <c r="B41" s="23" t="n">
         <v>2021</v>
       </c>
-      <c r="C41" s="23" t="n">
+      <c r="C41" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="D41" s="23" t="n">
+      <c r="D41" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="E41" s="23" t="n"/>
-      <c r="F41" s="23" t="n"/>
-      <c r="G41" s="23" t="n"/>
-      <c r="H41" s="23" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="24" t="n"/>
+      <c r="G41" s="24" t="n"/>
+      <c r="H41" s="24" t="n"/>
       <c r="I41" s="1" t="n"/>
-      <c r="J41" s="22" t="n">
+      <c r="J41" s="23" t="n">
         <v>2021</v>
       </c>
-      <c r="K41" s="23" t="n">
+      <c r="K41" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="L41" s="23" t="n">
+      <c r="L41" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="M41" s="23" t="n"/>
-      <c r="N41" s="23" t="n"/>
-      <c r="O41" s="23" t="n"/>
-      <c r="P41" s="23" t="n"/>
+      <c r="M41" s="24" t="n"/>
+      <c r="N41" s="24" t="n"/>
+      <c r="O41" s="24" t="n"/>
+      <c r="P41" s="24" t="n"/>
     </row>
     <row r="42" ht="13" customHeight="1">
       <c r="A42" s="1" t="n"/>
-      <c r="B42" s="24" t="n">
+      <c r="B42" s="25" t="n">
         <v>2020</v>
       </c>
-      <c r="C42" s="25" t="n">
+      <c r="C42" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="D42" s="25" t="n">
+      <c r="D42" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="E42" s="25" t="n"/>
-      <c r="F42" s="25" t="n"/>
-      <c r="G42" s="25" t="n"/>
-      <c r="H42" s="25" t="n"/>
+      <c r="E42" s="26" t="n"/>
+      <c r="F42" s="26" t="n"/>
+      <c r="G42" s="26" t="n"/>
+      <c r="H42" s="26" t="n"/>
       <c r="I42" s="1" t="n"/>
-      <c r="J42" s="24" t="n">
+      <c r="J42" s="25" t="n">
         <v>2020</v>
       </c>
-      <c r="K42" s="25" t="n"/>
-      <c r="L42" s="25" t="n">
+      <c r="K42" s="26" t="n"/>
+      <c r="L42" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="M42" s="25" t="n"/>
-      <c r="N42" s="25" t="n"/>
-      <c r="O42" s="25" t="n"/>
-      <c r="P42" s="25" t="n"/>
+      <c r="M42" s="26" t="n"/>
+      <c r="N42" s="26" t="n"/>
+      <c r="O42" s="26" t="n"/>
+      <c r="P42" s="26" t="n"/>
     </row>
     <row r="43" ht="13" customHeight="1">
       <c r="A43" s="1" t="n"/>
-      <c r="B43" s="24" t="n">
+      <c r="B43" s="25" t="n">
         <v>2019</v>
       </c>
-      <c r="C43" s="25" t="n">
+      <c r="C43" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="D43" s="25" t="n">
+      <c r="D43" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="E43" s="25" t="n"/>
-      <c r="F43" s="25" t="n"/>
-      <c r="G43" s="25" t="n"/>
-      <c r="H43" s="25" t="n"/>
+      <c r="E43" s="26" t="n"/>
+      <c r="F43" s="26" t="n"/>
+      <c r="G43" s="26" t="n"/>
+      <c r="H43" s="26" t="n"/>
       <c r="I43" s="1" t="n"/>
-      <c r="J43" s="24" t="n">
+      <c r="J43" s="25" t="n">
         <v>2019</v>
       </c>
-      <c r="K43" s="25" t="n"/>
-      <c r="L43" s="25" t="n">
+      <c r="K43" s="26" t="n"/>
+      <c r="L43" s="26" t="n">
         <v>9</v>
       </c>
-      <c r="M43" s="25" t="n"/>
-      <c r="N43" s="25" t="n"/>
-      <c r="O43" s="25" t="n"/>
-      <c r="P43" s="25" t="n"/>
+      <c r="M43" s="26" t="n"/>
+      <c r="N43" s="26" t="n"/>
+      <c r="O43" s="26" t="n"/>
+      <c r="P43" s="26" t="n"/>
     </row>
     <row r="44" ht="13" customHeight="1">
       <c r="A44" s="1" t="n"/>
-      <c r="B44" s="24" t="n">
+      <c r="B44" s="25" t="n">
         <v>2018</v>
       </c>
-      <c r="C44" s="25" t="n">
+      <c r="C44" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D44" s="25" t="n"/>
-      <c r="E44" s="25" t="n"/>
-      <c r="F44" s="25" t="n"/>
-      <c r="G44" s="25" t="n"/>
-      <c r="H44" s="25" t="n"/>
+      <c r="D44" s="26" t="n"/>
+      <c r="E44" s="26" t="n"/>
+      <c r="F44" s="26" t="n"/>
+      <c r="G44" s="26" t="n"/>
+      <c r="H44" s="26" t="n"/>
       <c r="I44" s="1" t="n"/>
-      <c r="J44" s="24" t="n">
+      <c r="J44" s="25" t="n">
         <v>2018</v>
       </c>
-      <c r="K44" s="25" t="n"/>
-      <c r="L44" s="25" t="n">
+      <c r="K44" s="26" t="n"/>
+      <c r="L44" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="M44" s="25" t="n"/>
-      <c r="N44" s="25" t="n"/>
-      <c r="O44" s="25" t="n"/>
-      <c r="P44" s="25" t="n"/>
+      <c r="M44" s="26" t="n"/>
+      <c r="N44" s="26" t="n"/>
+      <c r="O44" s="26" t="n"/>
+      <c r="P44" s="26" t="n"/>
     </row>
     <row r="45" ht="13" customHeight="1">
       <c r="A45" s="1" t="n"/>
-      <c r="B45" s="24" t="n">
+      <c r="B45" s="25" t="n">
         <v>2017</v>
       </c>
-      <c r="C45" s="25" t="n">
+      <c r="C45" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D45" s="25" t="n">
+      <c r="D45" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E45" s="25" t="n"/>
-      <c r="F45" s="25" t="n"/>
-      <c r="G45" s="25" t="n"/>
-      <c r="H45" s="25" t="n"/>
+      <c r="E45" s="26" t="n"/>
+      <c r="F45" s="26" t="n"/>
+      <c r="G45" s="26" t="n"/>
+      <c r="H45" s="26" t="n"/>
       <c r="I45" s="1" t="n"/>
-      <c r="J45" s="24" t="n">
+      <c r="J45" s="25" t="n">
         <v>2017</v>
       </c>
-      <c r="K45" s="25" t="n">
+      <c r="K45" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="L45" s="25" t="n"/>
-      <c r="M45" s="25" t="n"/>
-      <c r="N45" s="25" t="n"/>
-      <c r="O45" s="25" t="n"/>
-      <c r="P45" s="25" t="n"/>
+      <c r="L45" s="26" t="n"/>
+      <c r="M45" s="26" t="n"/>
+      <c r="N45" s="26" t="n"/>
+      <c r="O45" s="26" t="n"/>
+      <c r="P45" s="26" t="n"/>
     </row>
     <row r="46" ht="13" customHeight="1">
       <c r="A46" s="1" t="n"/>
-      <c r="B46" s="24" t="n">
+      <c r="B46" s="25" t="n">
         <v>2016</v>
       </c>
-      <c r="C46" s="25" t="n">
+      <c r="C46" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D46" s="25" t="n"/>
-      <c r="E46" s="25" t="n"/>
-      <c r="F46" s="25" t="n"/>
-      <c r="G46" s="25" t="n"/>
-      <c r="H46" s="25" t="n"/>
+      <c r="D46" s="26" t="n"/>
+      <c r="E46" s="26" t="n"/>
+      <c r="F46" s="26" t="n"/>
+      <c r="G46" s="26" t="n"/>
+      <c r="H46" s="26" t="n"/>
       <c r="I46" s="1" t="n"/>
-      <c r="J46" s="24" t="n">
+      <c r="J46" s="25" t="n">
         <v>2016</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="K46" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="L46" s="25" t="n">
+      <c r="L46" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="M46" s="25" t="n"/>
-      <c r="N46" s="25" t="n"/>
-      <c r="O46" s="25" t="n"/>
-      <c r="P46" s="25" t="n"/>
+      <c r="M46" s="26" t="n"/>
+      <c r="N46" s="26" t="n"/>
+      <c r="O46" s="26" t="n"/>
+      <c r="P46" s="26" t="n"/>
     </row>
     <row r="47" ht="13" customHeight="1">
       <c r="A47" s="1" t="n"/>
-      <c r="B47" s="26" t="n">
+      <c r="B47" s="27" t="n">
         <v>2015</v>
       </c>
-      <c r="C47" s="27" t="n"/>
-      <c r="D47" s="27" t="n"/>
-      <c r="E47" s="27" t="n"/>
-      <c r="F47" s="27" t="n"/>
-      <c r="G47" s="27" t="n"/>
-      <c r="H47" s="27" t="n"/>
+      <c r="C47" s="28" t="n"/>
+      <c r="D47" s="28" t="n"/>
+      <c r="E47" s="28" t="n"/>
+      <c r="F47" s="28" t="n"/>
+      <c r="G47" s="28" t="n"/>
+      <c r="H47" s="28" t="n"/>
       <c r="I47" s="1" t="n"/>
-      <c r="J47" s="26" t="n">
+      <c r="J47" s="27" t="n">
         <v>2015</v>
       </c>
-      <c r="K47" s="27" t="n"/>
-      <c r="L47" s="27" t="n">
+      <c r="K47" s="28" t="n"/>
+      <c r="L47" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="M47" s="27" t="n"/>
-      <c r="N47" s="27" t="n"/>
-      <c r="O47" s="27" t="n"/>
-      <c r="P47" s="27" t="n"/>
+      <c r="M47" s="28" t="n"/>
+      <c r="N47" s="28" t="n"/>
+      <c r="O47" s="28" t="n"/>
+      <c r="P47" s="28" t="n"/>
     </row>
     <row r="48" ht="13" customHeight="1">
       <c r="A48" s="1" t="n"/>
-      <c r="B48" s="26" t="n">
+      <c r="B48" s="27" t="n">
         <v>2014</v>
       </c>
-      <c r="C48" s="27" t="n">
+      <c r="C48" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="D48" s="27" t="n"/>
-      <c r="E48" s="27" t="n"/>
-      <c r="F48" s="27" t="n"/>
-      <c r="G48" s="27" t="n"/>
-      <c r="H48" s="27" t="n"/>
+      <c r="D48" s="28" t="n"/>
+      <c r="E48" s="28" t="n"/>
+      <c r="F48" s="28" t="n"/>
+      <c r="G48" s="28" t="n"/>
+      <c r="H48" s="28" t="n"/>
       <c r="I48" s="1" t="n"/>
-      <c r="J48" s="26" t="n">
+      <c r="J48" s="27" t="n">
         <v>2014</v>
       </c>
-      <c r="K48" s="27" t="n"/>
-      <c r="L48" s="27" t="n">
+      <c r="K48" s="28" t="n"/>
+      <c r="L48" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="M48" s="27" t="n"/>
-      <c r="N48" s="27" t="n"/>
-      <c r="O48" s="27" t="n"/>
-      <c r="P48" s="27" t="n"/>
+      <c r="M48" s="28" t="n"/>
+      <c r="N48" s="28" t="n"/>
+      <c r="O48" s="28" t="n"/>
+      <c r="P48" s="28" t="n"/>
     </row>
     <row r="49" ht="13" customHeight="1">
       <c r="A49" s="1" t="n"/>
-      <c r="B49" s="26" t="n">
+      <c r="B49" s="27" t="n">
         <v>2013</v>
       </c>
-      <c r="C49" s="27" t="n">
+      <c r="C49" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="D49" s="27" t="n"/>
-      <c r="E49" s="27" t="n">
+      <c r="D49" s="28" t="n"/>
+      <c r="E49" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="F49" s="27" t="n">
+      <c r="F49" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="G49" s="27" t="n">
+      <c r="G49" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="H49" s="27" t="n"/>
+      <c r="H49" s="28" t="n"/>
       <c r="I49" s="1" t="n"/>
-      <c r="J49" s="26" t="n">
+      <c r="J49" s="27" t="n">
         <v>2013</v>
       </c>
-      <c r="K49" s="27" t="n"/>
-      <c r="L49" s="27" t="n"/>
-      <c r="M49" s="27" t="n">
+      <c r="K49" s="28" t="n"/>
+      <c r="L49" s="28" t="n"/>
+      <c r="M49" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="N49" s="27" t="n">
+      <c r="N49" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="O49" s="27" t="n"/>
-      <c r="P49" s="27" t="n"/>
+      <c r="O49" s="28" t="n"/>
+      <c r="P49" s="28" t="n"/>
     </row>
     <row r="50" ht="13" customHeight="1">
       <c r="A50" s="1" t="n"/>
-      <c r="B50" s="26" t="n">
+      <c r="B50" s="27" t="n">
         <v>2012</v>
       </c>
-      <c r="C50" s="27" t="n">
+      <c r="C50" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="D50" s="27" t="n"/>
-      <c r="E50" s="27" t="n"/>
-      <c r="F50" s="27" t="n"/>
-      <c r="G50" s="27" t="n"/>
-      <c r="H50" s="27" t="n"/>
+      <c r="D50" s="28" t="n"/>
+      <c r="E50" s="28" t="n"/>
+      <c r="F50" s="28" t="n"/>
+      <c r="G50" s="28" t="n"/>
+      <c r="H50" s="28" t="n"/>
       <c r="I50" s="1" t="n"/>
-      <c r="J50" s="26" t="n">
+      <c r="J50" s="27" t="n">
         <v>2012</v>
       </c>
-      <c r="K50" s="27" t="n"/>
-      <c r="L50" s="27" t="n">
+      <c r="K50" s="28" t="n"/>
+      <c r="L50" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="M50" s="27" t="n">
+      <c r="M50" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="N50" s="27" t="n"/>
-      <c r="O50" s="27" t="n"/>
-      <c r="P50" s="27" t="n"/>
+      <c r="N50" s="28" t="n"/>
+      <c r="O50" s="28" t="n"/>
+      <c r="P50" s="28" t="n"/>
     </row>
     <row r="51" ht="13" customHeight="1">
       <c r="A51" s="1" t="n"/>
-      <c r="B51" s="26" t="n">
+      <c r="B51" s="27" t="n">
         <v>2011</v>
       </c>
-      <c r="C51" s="27" t="n"/>
-      <c r="D51" s="27" t="n"/>
-      <c r="E51" s="27" t="n"/>
-      <c r="F51" s="27" t="n"/>
-      <c r="G51" s="27" t="n"/>
-      <c r="H51" s="27" t="n"/>
+      <c r="C51" s="28" t="n"/>
+      <c r="D51" s="28" t="n"/>
+      <c r="E51" s="28" t="n"/>
+      <c r="F51" s="28" t="n"/>
+      <c r="G51" s="28" t="n"/>
+      <c r="H51" s="28" t="n"/>
       <c r="I51" s="1" t="n"/>
-      <c r="J51" s="26" t="n">
+      <c r="J51" s="27" t="n">
         <v>2011</v>
       </c>
-      <c r="K51" s="27" t="n"/>
-      <c r="L51" s="27" t="n"/>
-      <c r="M51" s="27" t="n"/>
-      <c r="N51" s="27" t="n">
+      <c r="K51" s="28" t="n"/>
+      <c r="L51" s="28" t="n"/>
+      <c r="M51" s="28" t="n"/>
+      <c r="N51" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="O51" s="27" t="n"/>
-      <c r="P51" s="27" t="n"/>
+      <c r="O51" s="28" t="n"/>
+      <c r="P51" s="28" t="n"/>
     </row>
     <row r="52" ht="13" customHeight="1">
       <c r="A52" s="1" t="n"/>
-      <c r="B52" s="28" t="n">
+      <c r="B52" s="29" t="n">
         <v>2010</v>
       </c>
-      <c r="C52" s="29" t="n"/>
-      <c r="D52" s="29" t="n"/>
-      <c r="E52" s="29" t="n"/>
-      <c r="F52" s="29" t="n"/>
-      <c r="G52" s="29" t="n"/>
-      <c r="H52" s="29" t="n"/>
+      <c r="C52" s="30" t="n"/>
+      <c r="D52" s="30" t="n"/>
+      <c r="E52" s="30" t="n"/>
+      <c r="F52" s="30" t="n"/>
+      <c r="G52" s="30" t="n"/>
+      <c r="H52" s="30" t="n"/>
       <c r="I52" s="1" t="n"/>
-      <c r="J52" s="28" t="n">
+      <c r="J52" s="29" t="n">
         <v>2010</v>
       </c>
-      <c r="K52" s="29" t="n"/>
-      <c r="L52" s="29" t="n"/>
-      <c r="M52" s="29" t="n"/>
-      <c r="N52" s="29" t="n"/>
-      <c r="O52" s="29" t="n"/>
-      <c r="P52" s="29" t="n"/>
+      <c r="K52" s="30" t="n"/>
+      <c r="L52" s="30" t="n"/>
+      <c r="M52" s="30" t="n"/>
+      <c r="N52" s="30" t="n"/>
+      <c r="O52" s="30" t="n"/>
+      <c r="P52" s="30" t="n"/>
     </row>
     <row r="53" ht="13" customHeight="1">
       <c r="A53" s="1" t="n"/>
-      <c r="B53" s="30" t="inlineStr">
+      <c r="B53" s="13" t="inlineStr">
         <is>
           <t>GTTL</t>
         </is>
       </c>
-      <c r="C53" s="30" t="n">
+      <c r="C53" s="13" t="n">
         <v>18</v>
       </c>
-      <c r="D53" s="30" t="n">
+      <c r="D53" s="13" t="n">
         <v>19</v>
       </c>
-      <c r="E53" s="30" t="n">
+      <c r="E53" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="F53" s="30" t="n">
+      <c r="F53" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G53" s="30" t="n">
+      <c r="G53" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H53" s="30" t="n"/>
+      <c r="H53" s="13" t="n"/>
       <c r="I53" s="1" t="n"/>
-      <c r="J53" s="30" t="inlineStr">
+      <c r="J53" s="13" t="inlineStr">
         <is>
           <t>GTTL</t>
         </is>
       </c>
-      <c r="K53" s="30" t="n">
+      <c r="K53" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="L53" s="30" t="n">
+      <c r="L53" s="13" t="n">
         <v>42</v>
       </c>
-      <c r="M53" s="30" t="n">
+      <c r="M53" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="N53" s="30" t="n">
+      <c r="N53" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="O53" s="30" t="n"/>
-      <c r="P53" s="30" t="n"/>
+      <c r="O53" s="13" t="n"/>
+      <c r="P53" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -5323,8 +5443,8 @@
         <f>'TOTAL RH'!B2</f>
         <v/>
       </c>
-      <c r="C9" s="53" t="n"/>
-      <c r="D9" s="54" t="n"/>
+      <c r="C9" s="56" t="n"/>
+      <c r="D9" s="57" t="n"/>
       <c r="E9" s="1" t="n"/>
       <c r="F9" s="1" t="n"/>
       <c r="G9" s="1" t="n"/>
@@ -5332,8 +5452,8 @@
         <f>'TOTAL RH'!H2</f>
         <v/>
       </c>
-      <c r="I9" s="53" t="n"/>
-      <c r="J9" s="54" t="n"/>
+      <c r="I9" s="56" t="n"/>
+      <c r="J9" s="57" t="n"/>
       <c r="K9" s="1" t="n"/>
       <c r="L9" s="1" t="n"/>
       <c r="M9" s="1" t="n"/>
@@ -5529,7 +5649,7 @@
         <f>'TOTAL RH'!C8</f>
         <v/>
       </c>
-      <c r="D15" s="55">
+      <c r="D15" s="58">
         <f>'TOTAL RH'!D8</f>
         <v/>
       </c>
@@ -5601,7 +5721,7 @@
         <f>'TOTAL RH'!C10</f>
         <v/>
       </c>
-      <c r="D17" s="55">
+      <c r="D17" s="58">
         <f>'TOTAL RH'!D10</f>
         <v/>
       </c>
@@ -5673,7 +5793,7 @@
         <f>'TOTAL RH'!C12</f>
         <v/>
       </c>
-      <c r="D19" s="55">
+      <c r="D19" s="58">
         <f>'TOTAL RH'!D12</f>
         <v/>
       </c>
@@ -5688,7 +5808,7 @@
         <f>'TOTAL RH'!I12</f>
         <v/>
       </c>
-      <c r="J19" s="55">
+      <c r="J19" s="58">
         <f>'TOTAL RH'!J12</f>
         <v/>
       </c>
@@ -5763,8 +5883,8 @@
         <f>'TOTAL RH'!B2</f>
         <v/>
       </c>
-      <c r="C23" s="53" t="n"/>
-      <c r="D23" s="54" t="n"/>
+      <c r="C23" s="56" t="n"/>
+      <c r="D23" s="57" t="n"/>
       <c r="E23" s="1" t="n"/>
       <c r="F23" s="1" t="n"/>
       <c r="G23" s="1" t="n"/>
@@ -5772,8 +5892,8 @@
         <f>'TOTAL RH'!H2</f>
         <v/>
       </c>
-      <c r="I23" s="53" t="n"/>
-      <c r="J23" s="54" t="n"/>
+      <c r="I23" s="56" t="n"/>
+      <c r="J23" s="57" t="n"/>
       <c r="K23" s="1" t="n"/>
       <c r="L23" s="1" t="n"/>
       <c r="M23" s="1" t="n"/>
@@ -6061,8 +6181,8 @@
           <t>BKK27 current mix</t>
         </is>
       </c>
-      <c r="C34" s="53" t="n"/>
-      <c r="D34" s="54" t="n"/>
+      <c r="C34" s="56" t="n"/>
+      <c r="D34" s="57" t="n"/>
       <c r="E34" s="1" t="n"/>
       <c r="F34" s="1" t="n"/>
       <c r="G34" s="1" t="n"/>
@@ -6071,8 +6191,8 @@
           <t>LCH27 current mix</t>
         </is>
       </c>
-      <c r="I34" s="53" t="n"/>
-      <c r="J34" s="54" t="n"/>
+      <c r="I34" s="56" t="n"/>
+      <c r="J34" s="57" t="n"/>
       <c r="K34" s="1" t="n"/>
       <c r="L34" s="1" t="n"/>
       <c r="M34" s="1" t="n"/>

</xml_diff>